<commit_message>
Add DOIs for 85 publications
Looked up in Crossref and accepted only when the title, year and
journal or first author matched, or (for 12 harder cases) when the
journal, volume and first page matched exactly. All 98 publications
now link to their DOI.
</commit_message>
<xml_diff>
--- a/content/lab-content.xlsx
+++ b/content/lab-content.xlsx
@@ -370,7 +370,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1377" uniqueCount="796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1462" uniqueCount="881">
   <si>
     <t>Lab website content</t>
   </si>
@@ -1781,6 +1781,9 @@
     <t>13(4), bio060415</t>
   </si>
   <si>
+    <t>10.1242/bio.060415</t>
+  </si>
+  <si>
     <t>https://journals.biologists.com/bio/article/13/4/bio060415/347005/SRRM2-splicing-factor-modulates-cell-fate-in-early</t>
   </si>
   <si>
@@ -1796,6 +1799,9 @@
     <t>84(3), 415–428</t>
   </si>
   <si>
+    <t>10.1016/j.molcel.2023.12.032</t>
+  </si>
+  <si>
     <t>A single dose of cocaine rewires the 3D genome structure of midbrain dopamine neurons</t>
   </si>
   <si>
@@ -1841,6 +1847,9 @@
     <t>20, 993–994</t>
   </si>
   <si>
+    <t>10.1038/s41592-023-01905-z</t>
+  </si>
+  <si>
     <t>Multiplex-GAM: genome-wide identification of chromatin contacts yields insights overlooked by Hi-C</t>
   </si>
   <si>
@@ -1865,6 +1874,9 @@
     <t>32, 100443</t>
   </si>
   <si>
+    <t>10.1016/j.coisb.2022.100443</t>
+  </si>
+  <si>
     <t>A noncoding single-nucleotide polymorphism at 8q24 drives IDH1-mutant glioma formation</t>
   </si>
   <si>
@@ -1877,6 +1889,9 @@
     <t>378(6615), 68–78</t>
   </si>
   <si>
+    <t>10.1126/science.abj2890</t>
+  </si>
+  <si>
     <t>Single-cell-resolved dynamics of chromatin architecture delineate cell and regulatory states in zebrafish embryos</t>
   </si>
   <si>
@@ -1889,6 +1904,9 @@
     <t>2(1)</t>
   </si>
   <si>
+    <t>10.1016/j.xgen.2021.100083</t>
+  </si>
+  <si>
     <t>Altered nuclear architecture in blood cells from Huntington’s disease patients</t>
   </si>
   <si>
@@ -1901,6 +1919,9 @@
     <t>43(1), 379–385</t>
   </si>
   <si>
+    <t>10.1007/s10072-021-05289-w</t>
+  </si>
+  <si>
     <t>GAMIBHEAR: whole-genome haplotype reconstruction from Genome Architecture Mapping data</t>
   </si>
   <si>
@@ -1913,6 +1934,9 @@
     <t>37(19), 3128–3135</t>
   </si>
   <si>
+    <t>10.1093/bioinformatics/btab238</t>
+  </si>
+  <si>
     <t>Cell-type specialization is encoded by specific chromatin topologies</t>
   </si>
   <si>
@@ -1934,6 +1958,9 @@
     <t>18(5), 482–490</t>
   </si>
   <si>
+    <t>10.1038/s41592-021-01135-1</t>
+  </si>
+  <si>
     <t>The dynamics of chromatin architecture in brain development and function</t>
   </si>
   <si>
@@ -1946,6 +1973,9 @@
     <t>67, 84–93</t>
   </si>
   <si>
+    <t>10.1016/j.gde.2020.12.008</t>
+  </si>
+  <si>
     <t>LifeTime and improving European healthcare through cell-based interceptive medicine</t>
   </si>
   <si>
@@ -1955,6 +1985,9 @@
     <t>587(7834), 377–386</t>
   </si>
   <si>
+    <t>10.1038/s41586-020-2715-9</t>
+  </si>
+  <si>
     <t>Inference of chromosome 3D structures from GAM data by a physics computational approach</t>
   </si>
   <si>
@@ -1967,6 +2000,9 @@
     <t>181, 70–79</t>
   </si>
   <si>
+    <t>10.1016/j.ymeth.2019.09.018</t>
+  </si>
+  <si>
     <t>Evolving methodologies and concepts in 4D nucleome research</t>
   </si>
   <si>
@@ -1979,6 +2015,9 @@
     <t>64, 105–111</t>
   </si>
   <si>
+    <t>10.1016/j.ceb.2020.04.005</t>
+  </si>
+  <si>
     <t>Methods for mapping 3D chromosome architecture</t>
   </si>
   <si>
@@ -1991,6 +2030,9 @@
     <t>21(4), 207–226</t>
   </si>
   <si>
+    <t>10.1038/s41576-019-0195-2</t>
+  </si>
+  <si>
     <t>Editorial overview: Genome architecture and expression</t>
   </si>
   <si>
@@ -2003,6 +2045,9 @@
     <t>55, iii–iv</t>
   </si>
   <si>
+    <t>10.1016/j.gde.2019.09.001</t>
+  </si>
+  <si>
     <t>R-loops enhance polycomb repression at a subset of developmental regulator genes</t>
   </si>
   <si>
@@ -2012,6 +2057,9 @@
     <t>73(5), 930–945.e4</t>
   </si>
   <si>
+    <t>10.1016/j.molcel.2018.12.016</t>
+  </si>
+  <si>
     <t>Challenges and guidelines toward 4D nucleome data and model standards</t>
   </si>
   <si>
@@ -2024,6 +2072,9 @@
     <t>50(10), 1352–1358</t>
   </si>
   <si>
+    <t>10.1038/s41588-018-0236-3</t>
+  </si>
+  <si>
     <t>Polymer physics predicts the effects of structural variants on chromatin architecture</t>
   </si>
   <si>
@@ -2033,6 +2084,9 @@
     <t>50(5), 662–667</t>
   </si>
   <si>
+    <t>10.1038/s41588-018-0098-8</t>
+  </si>
+  <si>
     <t>RNA polymerase II primes Polycomb-repressed developmental genes throughout terminal neuronal differentiation</t>
   </si>
   <si>
@@ -2042,6 +2096,9 @@
     <t>13(10), MSB177754</t>
   </si>
   <si>
+    <t>10.15252/msb.20177754</t>
+  </si>
+  <si>
     <t>FANTOM5 CAGE profiles of human and mouse samples</t>
   </si>
   <si>
@@ -2054,6 +2111,9 @@
     <t>4(1), 170112</t>
   </si>
   <si>
+    <t>10.1038/sdata.2017.112</t>
+  </si>
+  <si>
     <t>Cell cycle: Continuous chromatin changes</t>
   </si>
   <si>
@@ -2063,6 +2123,9 @@
     <t>547(7661), 34</t>
   </si>
   <si>
+    <t>10.1038/547034a</t>
+  </si>
+  <si>
     <t>Flipping between Polycomb repressed and active transcriptional states introduces noise in gene expression</t>
   </si>
   <si>
@@ -2072,6 +2135,9 @@
     <t>8(1), 36</t>
   </si>
   <si>
+    <t>10.1038/s41467-017-00052-2</t>
+  </si>
+  <si>
     <t>Active and poised promoter states drive folding of the extended HoxB locus in mouse embryonic stem cells</t>
   </si>
   <si>
@@ -2084,6 +2150,9 @@
     <t>24(6), 515–524</t>
   </si>
   <si>
+    <t>10.1038/nsmb.3402</t>
+  </si>
+  <si>
     <t>Keep them close: PRC2 poises enhancer-promoter interactions at anterior neuronal genes</t>
   </si>
   <si>
@@ -2096,6 +2165,9 @@
     <t>20(5), 573–575</t>
   </si>
   <si>
+    <t>10.1016/j.stem.2017.04.006</t>
+  </si>
+  <si>
     <t>Maternal immune activation results in complex microglial transcriptome signature in the adult offspring that is reversed by minocycline treatment</t>
   </si>
   <si>
@@ -2108,6 +2180,9 @@
     <t>7(5), e1120</t>
   </si>
   <si>
+    <t>10.1038/tp.2017.80</t>
+  </si>
+  <si>
     <t>Complex multi-enhancer contacts captured by genome architecture mapping</t>
   </si>
   <si>
@@ -2117,6 +2192,9 @@
     <t>543(7646), 519–524</t>
   </si>
   <si>
+    <t>10.1038/nature21411</t>
+  </si>
+  <si>
     <t>A finer print than TADs: PRC1-mediated domains</t>
   </si>
   <si>
@@ -2126,6 +2204,9 @@
     <t>65(3), 373–375</t>
   </si>
   <si>
+    <t>10.1016/j.molcel.2017.01.028</t>
+  </si>
+  <si>
     <t>Examining topological domain influence on enhancer function</t>
   </si>
   <si>
@@ -2135,6 +2216,9 @@
     <t>39(5), 523–524</t>
   </si>
   <si>
+    <t>10.1016/j.devcel.2016.11.011</t>
+  </si>
+  <si>
     <t>Formation of new chromatin domains determines pathogenicity of genomic duplications</t>
   </si>
   <si>
@@ -2144,6 +2228,9 @@
     <t>538(7624), 265–269</t>
   </si>
   <si>
+    <t>10.1038/nature19800</t>
+  </si>
+  <si>
     <t>Gene activation by metazoan enhancers: diverse mechanisms stimulate distinct steps of transcription</t>
   </si>
   <si>
@@ -2153,6 +2240,9 @@
     <t>38(9), 881–893</t>
   </si>
   <si>
+    <t>10.1002/bies.201600032</t>
+  </si>
+  <si>
     <t>Mechanical regulation of transcription controls Polycomb-mediated gene silencing during lineage commitment</t>
   </si>
   <si>
@@ -2165,6 +2255,9 @@
     <t>18(8), 864–875</t>
   </si>
   <si>
+    <t>10.1038/ncb3387</t>
+  </si>
+  <si>
     <t>Methylation of RNA polymerase II non-consensus Lysine residues marks early transcription in mammalian cells</t>
   </si>
   <si>
@@ -2177,6 +2270,9 @@
     <t>4, e11215</t>
   </si>
   <si>
+    <t>10.7554/elife.11215</t>
+  </si>
+  <si>
     <t>Hierarchical folding and reorganization of chromosomes are linked to transcriptional changes in cellular differentiation</t>
   </si>
   <si>
@@ -2186,6 +2282,9 @@
     <t>11(12), MSB156492</t>
   </si>
   <si>
+    <t>10.15252/msb.20156492</t>
+  </si>
+  <si>
     <t>Polymer models of the organization of chromosomes in the nucleus of cells</t>
   </si>
   <si>
@@ -2198,6 +2297,9 @@
     <t>29(09), 1530003</t>
   </si>
   <si>
+    <t>10.1142/s0217984915300033</t>
+  </si>
+  <si>
     <t>Three-dimensional genome architecture: players and mechanisms</t>
   </si>
   <si>
@@ -2210,6 +2312,9 @@
     <t>16(4), 245–257</t>
   </si>
   <si>
+    <t>10.1038/nrm3965</t>
+  </si>
+  <si>
     <t>Transcribed enhancers lead waves of coordinated transcription in transitioning mammalian cells</t>
   </si>
   <si>
@@ -2219,6 +2324,9 @@
     <t>347(6225), 1010–1014</t>
   </si>
   <si>
+    <t>10.1126/science.1259418</t>
+  </si>
+  <si>
     <t>Stem cell epigenetics: looking forward</t>
   </si>
   <si>
@@ -2228,6 +2336,9 @@
     <t>14(6), 706–709</t>
   </si>
   <si>
+    <t>10.1016/j.stem.2014.05.011</t>
+  </si>
+  <si>
     <t>Models of chromosome structure</t>
   </si>
   <si>
@@ -2237,6 +2348,9 @@
     <t>28, 90–95</t>
   </si>
   <si>
+    <t>10.1016/j.ceb.2014.04.004</t>
+  </si>
+  <si>
     <t>Physical mechanisms behind the large scale features of chromatin organization</t>
   </si>
   <si>
@@ -2249,6 +2363,9 @@
     <t>5(2), e28447</t>
   </si>
   <si>
+    <t>10.4161/trns.28447</t>
+  </si>
+  <si>
     <t>An H3K9/S10 methyl-phospho switch modulates Polycomb and Pol II binding at repressed genes during differentiation</t>
   </si>
   <si>
@@ -2261,6 +2378,9 @@
     <t>25(6), 904–915</t>
   </si>
   <si>
+    <t>10.1091/mbc.e13-10-0628</t>
+  </si>
+  <si>
     <t>Polymer physics, scaling and heterogeneity in the spatial organisation of chromosomes in the cell nucleus</t>
   </si>
   <si>
@@ -2273,6 +2393,9 @@
     <t>9(36), 8631–8635</t>
   </si>
   <si>
+    <t>10.1039/c3sm51436f</t>
+  </si>
+  <si>
     <t>A polymer model explains the complexity of large-scale chromatin folding</t>
   </si>
   <si>
@@ -2285,6 +2408,9 @@
     <t>4(4), 267–273</t>
   </si>
   <si>
+    <t>10.4161/nucl.25432</t>
+  </si>
+  <si>
     <t>Polymer models of chromatin organization</t>
   </si>
   <si>
@@ -2297,6 +2423,9 @@
     <t>4, 113</t>
   </si>
   <si>
+    <t>10.3389/fgene.2013.00113</t>
+  </si>
+  <si>
     <t>A model of the large-scale organization of chromatin</t>
   </si>
   <si>
@@ -2309,6 +2438,9 @@
     <t>41(2), 508–512</t>
   </si>
   <si>
+    <t>10.1042/bst20120238</t>
+  </si>
+  <si>
     <t>Mean expression of the X-chromosome is associated with neuronal density</t>
   </si>
   <si>
@@ -2321,12 +2453,18 @@
     <t>6, 161</t>
   </si>
   <si>
+    <t>10.3389/fnins.2012.00161</t>
+  </si>
+  <si>
     <t>Complexity of chromatin folding is captured by the strings and binders switch model</t>
   </si>
   <si>
     <t>109(40), 16173–16178</t>
   </si>
   <si>
+    <t>10.1073/pnas.1204799109</t>
+  </si>
+  <si>
     <t>Proteomic analysis of mitotic RNA polymerase II reveals novel interactors and association with proteins dysfunctional in disease</t>
   </si>
   <si>
@@ -2339,6 +2477,9 @@
     <t>11(6)</t>
   </si>
   <si>
+    <t>10.1074/mcp.M111.011767</t>
+  </si>
+  <si>
     <t>Code breaking: the RNAPII modification code in pluripotency</t>
   </si>
   <si>
@@ -2351,6 +2492,9 @@
     <t>11(7), 1267–1268</t>
   </si>
   <si>
+    <t>10.4161/cc.19990</t>
+  </si>
+  <si>
     <t>Polycomb associates genome-wide with a specific RNA polymerase II variant, and regulates metabolic genes in ESCs</t>
   </si>
   <si>
@@ -2360,6 +2504,9 @@
     <t>10(2), 157–170</t>
   </si>
   <si>
+    <t>10.1016/j.stem.2011.12.017</t>
+  </si>
+  <si>
     <t>Polycomb targets seek closest neighbours</t>
   </si>
   <si>
@@ -2372,6 +2519,9 @@
     <t>7(3), e1002031</t>
   </si>
   <si>
+    <t>10.1371/journal.pgen.1002031</t>
+  </si>
+  <si>
     <t>Nuclear cell biology</t>
   </si>
   <si>
@@ -2381,6 +2531,9 @@
     <t>22(6), 722–722</t>
   </si>
   <si>
+    <t>10.1091/mbc.e10-12-0966</t>
+  </si>
+  <si>
     <t>Ring1B and Suv39h1 delineate distinct chromatin states at bivalent genes during early mouse lineage commitment</t>
   </si>
   <si>
@@ -2393,6 +2546,9 @@
     <t>137(15), 2483–2492</t>
   </si>
   <si>
+    <t>10.1242/dev.048363</t>
+  </si>
+  <si>
     <t>Short RNAs are transcribed from repressed polycomb target genes and interact with polycomb repressive complex-2</t>
   </si>
   <si>
@@ -2402,6 +2558,9 @@
     <t>38(5), 675–688</t>
   </si>
   <si>
+    <t>10.1016/j.molcel.2010.03.019</t>
+  </si>
+  <si>
     <t>Gene positioning</t>
   </si>
   <si>
@@ -2414,6 +2573,9 @@
     <t>2(6), a000588</t>
   </si>
   <si>
+    <t>10.1101/cshperspect.a000588</t>
+  </si>
+  <si>
     <t>Jarid2 is a PRC2 component in embryonic stem cells required for multi-lineage differentiation and recruitment of PRC1 and RNA Polymerase II to developmental regulators</t>
   </si>
   <si>
@@ -2423,6 +2585,9 @@
     <t>12(6), 618–624</t>
   </si>
   <si>
+    <t>10.1038/ncb2065</t>
+  </si>
+  <si>
     <t>Nucleus and gene expression: the structure and function conundrum</t>
   </si>
   <si>
@@ -2432,6 +2597,9 @@
     <t>22(3), 269–270</t>
   </si>
   <si>
+    <t>10.1016/j.ceb.2010.04.010</t>
+  </si>
+  <si>
     <t>Poised transcription factories prime silent uPA gene prior to activation</t>
   </si>
   <si>
@@ -2444,6 +2612,9 @@
     <t>8(1), e1000270</t>
   </si>
   <si>
+    <t>10.1371/journal.pbio.1000270</t>
+  </si>
+  <si>
     <t>Nuclear architecture in stem cells</t>
   </si>
   <si>
@@ -2456,6 +2627,9 @@
     <t>695, 14–25</t>
   </si>
   <si>
+    <t>10.1007/978-1-4419-7037-4_2</t>
+  </si>
+  <si>
     <t>Measurement of replication structures at the nanometer scale using super-resolution light microscopy</t>
   </si>
   <si>
@@ -2468,6 +2642,9 @@
     <t>38(2), e8</t>
   </si>
   <si>
+    <t>10.1093/nar/gkp901</t>
+  </si>
+  <si>
     <t>The molecular basis for stability of heterochromatin-mediated silencing in mammals</t>
   </si>
   <si>
@@ -2480,6 +2657,9 @@
     <t>2(1), 14</t>
   </si>
   <si>
+    <t>10.1186/1756-8935-2-14</t>
+  </si>
+  <si>
     <t>Modifications of RNA polymerase II are pivotal in regulating gene expression states</t>
   </si>
   <si>
@@ -2489,6 +2669,9 @@
     <t>10(11), 1213</t>
   </si>
   <si>
+    <t>10.1038/embor.2009.221</t>
+  </si>
+  <si>
     <t>3D chromatin regulation of Sonic hedgehog in the limb buds</t>
   </si>
   <si>
@@ -2498,6 +2681,9 @@
     <t>16(1), 9–11</t>
   </si>
   <si>
+    <t>10.1016/j.devcel.2008.12.010</t>
+  </si>
+  <si>
     <t>Mechanisms regulating S phase progression in mammalian cells</t>
   </si>
   <si>
@@ -2510,6 +2696,9 @@
     <t>14(11), 4199–4213</t>
   </si>
   <si>
+    <t>10.2741/3523</t>
+  </si>
+  <si>
     <t>Eukaryotic gene regulation in three dimensions and its impact on genome evolution</t>
   </si>
   <si>
@@ -2519,6 +2708,9 @@
     <t>18(6), 571–582</t>
   </si>
   <si>
+    <t>10.1016/j.gde.2008.10.002</t>
+  </si>
+  <si>
     <t>Changes in chromosome organization during PHA-activation of resting human lymphocytes measured by cryo-FISH</t>
   </si>
   <si>
@@ -2531,6 +2723,9 @@
     <t>16(3), 413–426</t>
   </si>
   <si>
+    <t>10.1007/s10577-008-1230-x</t>
+  </si>
+  <si>
     <t>Transcription and chromatin organization of a housekeeping gene cluster containing an integrated β-globin locus control region</t>
   </si>
   <si>
@@ -2540,6 +2735,9 @@
     <t>4(3), e1000016</t>
   </si>
   <si>
+    <t>10.1371/journal.pgen.1000016</t>
+  </si>
+  <si>
     <t>Ring1-mediated ubiquitination of H2A restrains poised RNA polymerase II at bivalent genes in mouse ES cells</t>
   </si>
   <si>
@@ -2549,6 +2747,9 @@
     <t>9(12), 1428–1435</t>
   </si>
   <si>
+    <t>10.1038/ncb1663</t>
+  </si>
+  <si>
     <t>Functional organisation of the genome during interphase</t>
   </si>
   <si>
@@ -2558,6 +2759,9 @@
     <t>17(5), 451–455</t>
   </si>
   <si>
+    <t>10.1016/j.gde.2007.08.008</t>
+  </si>
+  <si>
     <t>Advances in imaging the interphase nucleus using thin cryosections</t>
   </si>
   <si>
@@ -2570,6 +2774,9 @@
     <t>128(2), 97–104</t>
   </si>
   <si>
+    <t>10.1007/s00418-007-0310-x</t>
+  </si>
+  <si>
     <t>Desmin immunolocalisation in autosomal dominant Emery-Dreifuss muscular dystrophy</t>
   </si>
   <si>
@@ -2582,6 +2789,9 @@
     <t>17(4), 297–305</t>
   </si>
   <si>
+    <t>10.1016/j.nmd.2007.01.003</t>
+  </si>
+  <si>
     <t>Chromosome organization: new facts, new models</t>
   </si>
   <si>
@@ -2594,12 +2804,18 @@
     <t>17(3), 127–134</t>
   </si>
   <si>
+    <t>10.1016/j.tcb.2006.12.006</t>
+  </si>
+  <si>
     <t>Intermingling of chromosome territories in interphase suggests role in translocations and transcription-dependent associations</t>
   </si>
   <si>
     <t>4(5), e138</t>
   </si>
   <si>
+    <t>10.1371/journal.pbio.0040138</t>
+  </si>
+  <si>
     <t>Splicing speckles are not reservoirs of RNA polymerase II, but contain an inactive form, phosphorylated on Serine2 residues of the C-terminal domain</t>
   </si>
   <si>
@@ -2609,6 +2825,9 @@
     <t>17(4), 1723–1733</t>
   </si>
   <si>
+    <t>10.1091/mbc.e05-08-0726</t>
+  </si>
+  <si>
     <t>Distribution of different phosphorylated forms of RNA polymerase II in relation to Cajal and PML bodies in human cells: an ultrastructural study</t>
   </si>
   <si>
@@ -2618,6 +2837,9 @@
     <t>125(1), 21–31</t>
   </si>
   <si>
+    <t>10.1007/s00418-005-0064-2</t>
+  </si>
+  <si>
     <t>Variant histone H3.3 marks promoters of transcriptionally active genes during mammalian cell division</t>
   </si>
   <si>
@@ -2627,6 +2849,9 @@
     <t>6(4), 354</t>
   </si>
   <si>
+    <t>10.1038/sj.embor.7400366</t>
+  </si>
+  <si>
     <t>Functional analysis of Vif protein shows less restriction of human immunodeficiency virus type 2 by APOBEC3G</t>
   </si>
   <si>
@@ -2639,6 +2864,9 @@
     <t>79(2), 823–833</t>
   </si>
   <si>
+    <t>10.1128/jvi.79.2.823-833.2005</t>
+  </si>
+  <si>
     <t>CD8α is an activation marker for a subset of peripheral CD4 T cells</t>
   </si>
   <si>
@@ -2651,6 +2879,9 @@
     <t>34(5), 1262–1271</t>
   </si>
   <si>
+    <t>10.1002/eji.200324363</t>
+  </si>
+  <si>
     <t>Fixation-induced redistribution of hyperphosphorylated RNA polymerase II in the nucleus of human cells</t>
   </si>
   <si>
@@ -2663,6 +2894,9 @@
     <t>295(2), 460–468</t>
   </si>
   <si>
+    <t>10.1016/j.yexcr.2004.01.020</t>
+  </si>
+  <si>
     <t>Measuring the size of biological nanostructures with spatially modulated illumination microscopy</t>
   </si>
   <si>
@@ -2672,6 +2906,9 @@
     <t>15(5), 2449–2455</t>
   </si>
   <si>
+    <t>10.1091/mbc.e04-01-0045</t>
+  </si>
+  <si>
     <t>Interaction of proteins with promoter elements of the human U2 snRNA genes in vivo</t>
   </si>
   <si>
@@ -2684,6 +2921,9 @@
     <t>315, 103–112</t>
   </si>
   <si>
+    <t>10.1016/s0378-1119(03)00717-0</t>
+  </si>
+  <si>
     <t>Transcription factories: quantitative studies of nanostructures in the mammalian nucleus</t>
   </si>
   <si>
@@ -2693,6 +2933,9 @@
     <t>11(5), 461–470</t>
   </si>
   <si>
+    <t>10.1023/a:1024926710797</t>
+  </si>
+  <si>
     <t>Genome function and nuclear architecture: from gene expression to nanoscience</t>
   </si>
   <si>
@@ -2705,6 +2948,9 @@
     <t>13(6a), 1029–1041</t>
   </si>
   <si>
+    <t>10.1101/gr.946403</t>
+  </si>
+  <si>
     <t>From linear genome sequence to three-dimensional organization of the cell nucleus</t>
   </si>
   <si>
@@ -2717,6 +2963,9 @@
     <t>4(3), 310</t>
   </si>
   <si>
+    <t>10.1186/gb-2003-4-3-310</t>
+  </si>
+  <si>
     <t>Cellular genomics: which genes are transcribed, when and where?</t>
   </si>
   <si>
@@ -2726,6 +2975,9 @@
     <t>28(1), 6–9</t>
   </si>
   <si>
+    <t>10.1016/s0968-0004(02)00011-7</t>
+  </si>
+  <si>
     <t>Genomics meets nanoscience: probing genes and the cell nucleus at 10−9 meters</t>
   </si>
   <si>
@@ -2733,6 +2985,9 @@
   </si>
   <si>
     <t>3(3), reports4007.1</t>
+  </si>
+  <si>
+    <t>10.1186/gb-2002-3-3-reports4007</t>
   </si>
   <si>
     <t>Inventors</t>
@@ -3424,16 +3679,16 @@
         <v>90</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>786</v>
+        <v>871</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>787</v>
+        <v>872</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>788</v>
+        <v>873</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>789</v>
+        <v>874</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>105</v>
@@ -3447,19 +3702,19 @@
         <v>2026</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>790</v>
+        <v>875</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>791</v>
+        <v>876</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>792</v>
+        <v>877</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>793</v>
+        <v>878</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>794</v>
+        <v>879</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2" t="s">
@@ -3471,19 +3726,19 @@
         <v>2025</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>790</v>
+        <v>875</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>791</v>
+        <v>876</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>792</v>
+        <v>877</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>795</v>
+        <v>880</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>794</v>
+        <v>879</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
@@ -6574,12 +6829,14 @@
       <c r="E10" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>468</v>
+      </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>131</v>
@@ -6593,18 +6850,20 @@
         <v>2024</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="F11" s="2"/>
+        <v>473</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>474</v>
+      </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -6621,17 +6880,17 @@
         <v>2024</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>438</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -6649,17 +6908,17 @@
         <v>2024</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -6677,17 +6936,17 @@
         <v>2024</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -6705,18 +6964,20 @@
         <v>2023</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>487</v>
-      </c>
-      <c r="F15" s="2"/>
+        <v>489</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>490</v>
+      </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -6733,19 +6994,19 @@
         <v>2023</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>489</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>486</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -6763,18 +7024,20 @@
         <v>2023</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="F17" s="2"/>
+        <v>498</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>499</v>
+      </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -6791,18 +7054,20 @@
         <v>2022</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="F18" s="2"/>
+        <v>503</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>504</v>
+      </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -6819,18 +7084,20 @@
         <v>2022</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>503</v>
-      </c>
-      <c r="F19" s="2"/>
+        <v>508</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>509</v>
+      </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -6847,18 +7114,20 @@
         <v>2022</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="F20" s="2"/>
+        <v>513</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>514</v>
+      </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -6875,18 +7144,20 @@
         <v>2021</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>511</v>
-      </c>
-      <c r="F21" s="2"/>
+        <v>518</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>519</v>
+      </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
@@ -6903,19 +7174,19 @@
         <v>2021</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>512</v>
+        <v>520</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>513</v>
+        <v>521</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>433</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>515</v>
+        <v>523</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -6933,18 +7204,20 @@
         <v>2021</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>516</v>
+        <v>524</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>517</v>
+        <v>525</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="F23" s="2"/>
+        <v>526</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>527</v>
+      </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -6961,18 +7234,20 @@
         <v>2021</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>519</v>
+        <v>528</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>520</v>
+        <v>529</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>522</v>
-      </c>
-      <c r="F24" s="2"/>
+        <v>531</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>532</v>
+      </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -6989,18 +7264,20 @@
         <v>2020</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>523</v>
+        <v>533</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>524</v>
+        <v>534</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>433</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>525</v>
-      </c>
-      <c r="F25" s="2"/>
+        <v>535</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>536</v>
+      </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
@@ -7017,18 +7294,20 @@
         <v>2020</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>529</v>
-      </c>
-      <c r="F26" s="2"/>
+        <v>540</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>541</v>
+      </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
@@ -7045,18 +7324,20 @@
         <v>2020</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>530</v>
+        <v>542</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>531</v>
+        <v>543</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>532</v>
+        <v>544</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F27" s="2"/>
+        <v>545</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>546</v>
+      </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
@@ -7073,18 +7354,20 @@
         <v>2020</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>534</v>
+        <v>547</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>535</v>
+        <v>548</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>536</v>
+        <v>549</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>537</v>
-      </c>
-      <c r="F28" s="2"/>
+        <v>550</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>551</v>
+      </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -7101,18 +7384,20 @@
         <v>2019</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>538</v>
+        <v>552</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>539</v>
+        <v>553</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>540</v>
+        <v>554</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>541</v>
-      </c>
-      <c r="F29" s="2"/>
+        <v>555</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>556</v>
+      </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
@@ -7129,18 +7414,20 @@
         <v>2019</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>542</v>
+        <v>557</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>543</v>
+        <v>558</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>544</v>
-      </c>
-      <c r="F30" s="2"/>
+        <v>559</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>560</v>
+      </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
@@ -7157,18 +7444,20 @@
         <v>2018</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>545</v>
+        <v>561</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>546</v>
+        <v>562</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F31" s="2"/>
+        <v>564</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>565</v>
+      </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -7185,18 +7474,20 @@
         <v>2018</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>549</v>
+        <v>566</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>547</v>
+        <v>563</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>551</v>
-      </c>
-      <c r="F32" s="2"/>
+        <v>568</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>569</v>
+      </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -7213,18 +7504,20 @@
         <v>2017</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>553</v>
+        <v>571</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>457</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>554</v>
-      </c>
-      <c r="F33" s="2"/>
+        <v>572</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>573</v>
+      </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -7241,18 +7534,20 @@
         <v>2017</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>555</v>
+        <v>574</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>556</v>
+        <v>575</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>557</v>
+        <v>576</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="F34" s="2"/>
+        <v>577</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>578</v>
+      </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -7269,18 +7564,20 @@
         <v>2017</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>559</v>
+        <v>579</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>560</v>
+        <v>580</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>433</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>561</v>
-      </c>
-      <c r="F35" s="2"/>
+        <v>581</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>582</v>
+      </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -7297,18 +7594,20 @@
         <v>2017</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>562</v>
+        <v>583</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>563</v>
+        <v>584</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="F36" s="2"/>
+        <v>585</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>586</v>
+      </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -7325,18 +7624,20 @@
         <v>2017</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>565</v>
+        <v>587</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>566</v>
+        <v>588</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>567</v>
+        <v>589</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>568</v>
-      </c>
-      <c r="F37" s="2"/>
+        <v>590</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>591</v>
+      </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -7353,18 +7654,20 @@
         <v>2017</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>569</v>
+        <v>592</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>570</v>
+        <v>593</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>571</v>
+        <v>594</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>572</v>
-      </c>
-      <c r="F38" s="2"/>
+        <v>595</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>596</v>
+      </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -7381,18 +7684,20 @@
         <v>2017</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>573</v>
+        <v>597</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>574</v>
+        <v>598</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>575</v>
+        <v>599</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>576</v>
-      </c>
-      <c r="F39" s="2"/>
+        <v>600</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>601</v>
+      </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
@@ -7409,18 +7714,20 @@
         <v>2017</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>577</v>
+        <v>602</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>578</v>
+        <v>603</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>433</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>579</v>
-      </c>
-      <c r="F40" s="2"/>
+        <v>604</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>605</v>
+      </c>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -7437,18 +7744,20 @@
         <v>2017</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>580</v>
+        <v>606</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>581</v>
+        <v>607</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="F41" s="2"/>
+        <v>608</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>609</v>
+      </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
@@ -7465,18 +7774,20 @@
         <v>2016</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>583</v>
+        <v>610</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>560</v>
+        <v>580</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>584</v>
+        <v>611</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="F42" s="2"/>
+        <v>612</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>613</v>
+      </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2"/>
@@ -7493,18 +7804,20 @@
         <v>2016</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>586</v>
+        <v>614</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>587</v>
+        <v>615</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>433</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="F43" s="2"/>
+        <v>616</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>617</v>
+      </c>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2"/>
@@ -7521,18 +7834,20 @@
         <v>2016</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>589</v>
+        <v>618</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>560</v>
+        <v>580</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>590</v>
+        <v>619</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>591</v>
-      </c>
-      <c r="F44" s="2"/>
+        <v>620</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>621</v>
+      </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2"/>
@@ -7549,18 +7864,20 @@
         <v>2016</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>592</v>
+        <v>622</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>593</v>
+        <v>623</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>594</v>
+        <v>624</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="F45" s="2"/>
+        <v>625</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>626</v>
+      </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
       <c r="I45" s="2"/>
@@ -7577,18 +7894,20 @@
         <v>2015</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>596</v>
+        <v>627</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>597</v>
+        <v>628</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>598</v>
+        <v>629</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="F46" s="2"/>
+        <v>630</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>631</v>
+      </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2"/>
@@ -7605,18 +7924,20 @@
         <v>2015</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>600</v>
+        <v>632</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>601</v>
+        <v>633</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>457</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="F47" s="2"/>
+        <v>634</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>635</v>
+      </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
       <c r="I47" s="2"/>
@@ -7633,18 +7954,20 @@
         <v>2015</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>603</v>
+        <v>636</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>604</v>
+        <v>637</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>605</v>
+        <v>638</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>606</v>
-      </c>
-      <c r="F48" s="2"/>
+        <v>639</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>640</v>
+      </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2"/>
@@ -7661,18 +7984,20 @@
         <v>2015</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>607</v>
+        <v>641</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>608</v>
+        <v>642</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>609</v>
+        <v>643</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>610</v>
-      </c>
-      <c r="F49" s="2"/>
+        <v>644</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>645</v>
+      </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
       <c r="I49" s="2"/>
@@ -7689,18 +8014,20 @@
         <v>2015</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>611</v>
+        <v>646</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>612</v>
+        <v>647</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>613</v>
-      </c>
-      <c r="F50" s="2"/>
+        <v>648</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>649</v>
+      </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2"/>
@@ -7717,18 +8044,20 @@
         <v>2014</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>614</v>
+        <v>650</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>615</v>
+        <v>651</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>571</v>
+        <v>594</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="F51" s="2"/>
+        <v>652</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>653</v>
+      </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
       <c r="I51" s="2"/>
@@ -7745,18 +8074,20 @@
         <v>2014</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>617</v>
+        <v>654</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>618</v>
+        <v>655</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>532</v>
+        <v>544</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>619</v>
-      </c>
-      <c r="F52" s="2"/>
+        <v>656</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>657</v>
+      </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="I52" s="2"/>
@@ -7773,18 +8104,20 @@
         <v>2014</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>620</v>
+        <v>658</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>621</v>
+        <v>659</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>622</v>
+        <v>660</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>623</v>
-      </c>
-      <c r="F53" s="2"/>
+        <v>661</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>662</v>
+      </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2"/>
@@ -7801,18 +8134,20 @@
         <v>2014</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>624</v>
+        <v>663</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>625</v>
+        <v>664</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>626</v>
+        <v>665</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="F54" s="2"/>
+        <v>666</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>667</v>
+      </c>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2"/>
@@ -7829,18 +8164,20 @@
         <v>2013</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>628</v>
+        <v>668</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>629</v>
+        <v>669</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>630</v>
+        <v>670</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>631</v>
-      </c>
-      <c r="F55" s="2"/>
+        <v>671</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>672</v>
+      </c>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2"/>
@@ -7857,18 +8194,20 @@
         <v>2013</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>632</v>
+        <v>673</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>633</v>
+        <v>674</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>634</v>
+        <v>675</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="F56" s="2"/>
+        <v>676</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>677</v>
+      </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
@@ -7885,18 +8224,20 @@
         <v>2013</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>636</v>
+        <v>678</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>637</v>
+        <v>679</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>638</v>
+        <v>680</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>639</v>
-      </c>
-      <c r="F57" s="2"/>
+        <v>681</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>682</v>
+      </c>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2"/>
@@ -7913,18 +8254,20 @@
         <v>2013</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>640</v>
+        <v>683</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>641</v>
+        <v>684</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>642</v>
+        <v>685</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>643</v>
-      </c>
-      <c r="F58" s="2"/>
+        <v>686</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>687</v>
+      </c>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
@@ -7941,18 +8284,20 @@
         <v>2012</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>644</v>
+        <v>688</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>645</v>
+        <v>689</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>646</v>
+        <v>690</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>647</v>
-      </c>
-      <c r="F59" s="2"/>
+        <v>691</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>692</v>
+      </c>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
@@ -7969,18 +8314,20 @@
         <v>2012</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>648</v>
+        <v>693</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>641</v>
+        <v>684</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>452</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>649</v>
-      </c>
-      <c r="F60" s="2"/>
+        <v>694</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>695</v>
+      </c>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
@@ -7997,18 +8344,20 @@
         <v>2012</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>650</v>
+        <v>696</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>651</v>
+        <v>697</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>652</v>
+        <v>698</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>653</v>
-      </c>
-      <c r="F61" s="2"/>
+        <v>699</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>700</v>
+      </c>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
@@ -8025,18 +8374,20 @@
         <v>2012</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>654</v>
+        <v>701</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>655</v>
+        <v>702</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>656</v>
+        <v>703</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>657</v>
-      </c>
-      <c r="F62" s="2"/>
+        <v>704</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>705</v>
+      </c>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
@@ -8053,18 +8404,20 @@
         <v>2012</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>658</v>
+        <v>706</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>659</v>
+        <v>707</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>571</v>
+        <v>594</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="F63" s="2"/>
+        <v>708</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>709</v>
+      </c>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2"/>
@@ -8081,18 +8434,20 @@
         <v>2011</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>661</v>
+        <v>710</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>662</v>
+        <v>711</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>663</v>
+        <v>712</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>664</v>
-      </c>
-      <c r="F64" s="2"/>
+        <v>713</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>714</v>
+      </c>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
@@ -8109,18 +8464,20 @@
         <v>2011</v>
       </c>
       <c r="B65" s="2" t="s">
+        <v>715</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>665</v>
       </c>
-      <c r="C65" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>626</v>
-      </c>
       <c r="E65" s="2" t="s">
-        <v>667</v>
-      </c>
-      <c r="F65" s="2"/>
+        <v>717</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>718</v>
+      </c>
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
@@ -8137,18 +8494,20 @@
         <v>2010</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>668</v>
+        <v>719</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>669</v>
+        <v>720</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>670</v>
+        <v>721</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>671</v>
-      </c>
-      <c r="F66" s="2"/>
+        <v>722</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>723</v>
+      </c>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2"/>
@@ -8165,18 +8524,20 @@
         <v>2010</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>672</v>
+        <v>724</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>673</v>
+        <v>725</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>674</v>
-      </c>
-      <c r="F67" s="2"/>
+        <v>726</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>727</v>
+      </c>
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
       <c r="I67" s="2"/>
@@ -8193,18 +8554,20 @@
         <v>2010</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>675</v>
+        <v>728</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>676</v>
+        <v>729</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>677</v>
+        <v>730</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="F68" s="2"/>
+        <v>731</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>732</v>
+      </c>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
       <c r="I68" s="2"/>
@@ -8221,18 +8584,20 @@
         <v>2010</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>679</v>
+        <v>733</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>680</v>
+        <v>734</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>594</v>
+        <v>624</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>681</v>
-      </c>
-      <c r="F69" s="2"/>
+        <v>735</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>736</v>
+      </c>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
       <c r="I69" s="2"/>
@@ -8249,18 +8614,20 @@
         <v>2010</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>682</v>
+        <v>737</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>683</v>
+        <v>738</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>532</v>
+        <v>544</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>684</v>
-      </c>
-      <c r="F70" s="2"/>
+        <v>739</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>740</v>
+      </c>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2"/>
@@ -8277,18 +8644,20 @@
         <v>2010</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>685</v>
+        <v>741</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>686</v>
+        <v>742</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>687</v>
+        <v>743</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>688</v>
-      </c>
-      <c r="F71" s="2"/>
+        <v>744</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>745</v>
+      </c>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2"/>
@@ -8305,18 +8674,20 @@
         <v>2010</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>689</v>
+        <v>746</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>690</v>
+        <v>747</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>691</v>
+        <v>748</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>692</v>
-      </c>
-      <c r="F72" s="2"/>
+        <v>749</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>750</v>
+      </c>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2"/>
@@ -8333,18 +8704,20 @@
         <v>2010</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>693</v>
+        <v>751</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>694</v>
+        <v>752</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>695</v>
+        <v>753</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>696</v>
-      </c>
-      <c r="F73" s="2"/>
+        <v>754</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>755</v>
+      </c>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2"/>
@@ -8361,18 +8734,20 @@
         <v>2009</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>697</v>
+        <v>756</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>698</v>
+        <v>757</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>699</v>
+        <v>758</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>700</v>
-      </c>
-      <c r="F74" s="2"/>
+        <v>759</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>760</v>
+      </c>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2"/>
@@ -8389,18 +8764,20 @@
         <v>2009</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>701</v>
+        <v>761</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>655</v>
+        <v>702</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>702</v>
+        <v>762</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>703</v>
-      </c>
-      <c r="F75" s="2"/>
+        <v>763</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>764</v>
+      </c>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
       <c r="I75" s="2"/>
@@ -8417,18 +8794,20 @@
         <v>2009</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>704</v>
+        <v>765</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>705</v>
+        <v>766</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>584</v>
+        <v>611</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>706</v>
-      </c>
-      <c r="F76" s="2"/>
+        <v>767</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>768</v>
+      </c>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2"/>
@@ -8445,18 +8824,20 @@
         <v>2009</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>707</v>
+        <v>769</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>708</v>
+        <v>770</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>709</v>
+        <v>771</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>710</v>
-      </c>
-      <c r="F77" s="2"/>
+        <v>772</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>773</v>
+      </c>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2"/>
@@ -8473,18 +8854,20 @@
         <v>2008</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>711</v>
+        <v>774</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>712</v>
+        <v>775</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>713</v>
-      </c>
-      <c r="F78" s="2"/>
+        <v>776</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>777</v>
+      </c>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2"/>
@@ -8501,18 +8884,20 @@
         <v>2008</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>714</v>
+        <v>778</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>715</v>
+        <v>779</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>716</v>
+        <v>780</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>717</v>
-      </c>
-      <c r="F79" s="2"/>
+        <v>781</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>782</v>
+      </c>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2"/>
@@ -8529,18 +8914,20 @@
         <v>2008</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>718</v>
+        <v>783</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>719</v>
+        <v>784</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>663</v>
+        <v>712</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>720</v>
-      </c>
-      <c r="F80" s="2"/>
+        <v>785</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>786</v>
+      </c>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2"/>
@@ -8557,18 +8944,20 @@
         <v>2007</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>721</v>
+        <v>787</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>722</v>
+        <v>788</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>594</v>
+        <v>624</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>723</v>
-      </c>
-      <c r="F81" s="2"/>
+        <v>789</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>790</v>
+      </c>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
       <c r="I81" s="2"/>
@@ -8585,18 +8974,20 @@
         <v>2007</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>724</v>
+        <v>791</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>725</v>
+        <v>792</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>726</v>
-      </c>
-      <c r="F82" s="2"/>
+        <v>793</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>794</v>
+      </c>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
       <c r="I82" s="2"/>
@@ -8613,18 +9004,20 @@
         <v>2007</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>727</v>
+        <v>795</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>728</v>
+        <v>796</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>729</v>
+        <v>797</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>730</v>
-      </c>
-      <c r="F83" s="2"/>
+        <v>798</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>799</v>
+      </c>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
       <c r="I83" s="2"/>
@@ -8641,18 +9034,20 @@
         <v>2007</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>731</v>
+        <v>800</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>732</v>
+        <v>801</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>733</v>
+        <v>802</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>734</v>
-      </c>
-      <c r="F84" s="2"/>
+        <v>803</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>804</v>
+      </c>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
       <c r="I84" s="2"/>
@@ -8669,18 +9064,20 @@
         <v>2007</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>735</v>
+        <v>805</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>736</v>
+        <v>806</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>737</v>
+        <v>807</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>738</v>
-      </c>
-      <c r="F85" s="2"/>
+        <v>808</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>809</v>
+      </c>
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
@@ -8697,18 +9094,20 @@
         <v>2006</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>739</v>
+        <v>810</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>736</v>
+        <v>806</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>687</v>
+        <v>743</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>740</v>
-      </c>
-      <c r="F86" s="2"/>
+        <v>811</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>812</v>
+      </c>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
@@ -8725,18 +9124,20 @@
         <v>2006</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>741</v>
+        <v>813</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>742</v>
+        <v>814</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>626</v>
+        <v>665</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>743</v>
-      </c>
-      <c r="F87" s="2"/>
+        <v>815</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>816</v>
+      </c>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
@@ -8753,18 +9154,20 @@
         <v>2006</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>744</v>
+        <v>817</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>745</v>
+        <v>818</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>729</v>
+        <v>797</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>746</v>
-      </c>
-      <c r="F88" s="2"/>
+        <v>819</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>820</v>
+      </c>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
@@ -8781,18 +9184,20 @@
         <v>2005</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>747</v>
+        <v>821</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>748</v>
+        <v>822</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>702</v>
+        <v>762</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>749</v>
-      </c>
-      <c r="F89" s="2"/>
+        <v>823</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>824</v>
+      </c>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
       <c r="I89" s="2"/>
@@ -8809,18 +9214,20 @@
         <v>2005</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>750</v>
+        <v>825</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>751</v>
+        <v>826</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>752</v>
+        <v>827</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>753</v>
-      </c>
-      <c r="F90" s="2"/>
+        <v>828</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>829</v>
+      </c>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
@@ -8837,18 +9244,20 @@
         <v>2004</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>754</v>
+        <v>830</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>755</v>
+        <v>831</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>756</v>
+        <v>832</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>757</v>
-      </c>
-      <c r="F91" s="2"/>
+        <v>833</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>834</v>
+      </c>
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
@@ -8865,18 +9274,20 @@
         <v>2004</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>758</v>
+        <v>835</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>759</v>
+        <v>836</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>760</v>
+        <v>837</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>761</v>
-      </c>
-      <c r="F92" s="2"/>
+        <v>838</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>839</v>
+      </c>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
       <c r="I92" s="2"/>
@@ -8893,18 +9304,20 @@
         <v>2004</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>762</v>
+        <v>840</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>763</v>
+        <v>841</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>626</v>
+        <v>665</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>764</v>
-      </c>
-      <c r="F93" s="2"/>
+        <v>842</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>843</v>
+      </c>
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2"/>
@@ -8921,18 +9334,20 @@
         <v>2003</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>765</v>
+        <v>844</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>766</v>
+        <v>845</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>767</v>
+        <v>846</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>768</v>
-      </c>
-      <c r="F94" s="2"/>
+        <v>847</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>848</v>
+      </c>
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
       <c r="I94" s="2"/>
@@ -8949,18 +9364,20 @@
         <v>2003</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>769</v>
+        <v>849</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>770</v>
+        <v>850</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>716</v>
+        <v>780</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>771</v>
-      </c>
-      <c r="F95" s="2"/>
+        <v>851</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>852</v>
+      </c>
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
       <c r="I95" s="2"/>
@@ -8977,18 +9394,20 @@
         <v>2003</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>772</v>
+        <v>853</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>773</v>
+        <v>854</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>774</v>
+        <v>855</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>775</v>
-      </c>
-      <c r="F96" s="2"/>
+        <v>856</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>857</v>
+      </c>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
       <c r="I96" s="2"/>
@@ -9005,18 +9424,20 @@
         <v>2003</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>776</v>
+        <v>858</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>777</v>
+        <v>859</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>778</v>
+        <v>860</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>779</v>
-      </c>
-      <c r="F97" s="2"/>
+        <v>861</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>862</v>
+      </c>
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
       <c r="I97" s="2"/>
@@ -9033,18 +9454,20 @@
         <v>2003</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>780</v>
+        <v>863</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>728</v>
+        <v>796</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>781</v>
+        <v>864</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>782</v>
-      </c>
-      <c r="F98" s="2"/>
+        <v>865</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>866</v>
+      </c>
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
       <c r="I98" s="2"/>
@@ -9061,18 +9484,20 @@
         <v>2003</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>783</v>
+        <v>867</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>784</v>
+        <v>868</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>778</v>
+        <v>860</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>785</v>
-      </c>
-      <c r="F99" s="2"/>
+        <v>869</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>870</v>
+      </c>
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
       <c r="I99" s="2"/>

</xml_diff>

<commit_message>
[Tweak] update member profiles
</commit_message>
<xml_diff>
--- a/content/lab-content.xlsx
+++ b/content/lab-content.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11004"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63B64FD-1801-C345-91E1-84BE9E28A631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{136F636E-F3EB-964B-A85B-6C2E9E49FCEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -748,7 +748,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1531" uniqueCount="933">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1532" uniqueCount="934">
   <si>
     <t>Lab website content</t>
   </si>
@@ -3551,6 +3551,9 @@
   </si>
   <si>
     <t>pela.jpg</t>
+  </si>
+  <si>
+    <t>jhe.jpg</t>
   </si>
 </sst>
 </file>
@@ -7774,6 +7777,9 @@
       <c r="F5" s="2" t="s">
         <v>189</v>
       </c>
+      <c r="G5" s="2" t="s">
+        <v>933</v>
+      </c>
       <c r="I5" s="2" t="s">
         <v>114</v>
       </c>

</xml_diff>

<commit_message>
[Check] test gallery and news
</commit_message>
<xml_diff>
--- a/content/lab-content.xlsx
+++ b/content/lab-content.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11011"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{568CEDB1-E95B-BC4E-B098-EAB9665C7024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50E69AA5-317F-764D-9E98-EDFAEB897BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="-20120" windowWidth="29920" windowHeight="18660" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2560" yWindow="-19640" windowWidth="29920" windowHeight="18660" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,9 @@
     <sheet name="Publications" sheetId="10" r:id="rId10"/>
     <sheet name="Patents" sheetId="11" r:id="rId11"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Gallery!$A$1:$F$9</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -746,7 +749,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1549" uniqueCount="937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="939">
   <si>
     <t>Lab website content</t>
   </si>
@@ -2087,12 +2090,6 @@
     <t>placeholder-1.svg</t>
   </si>
   <si>
-    <t>Lab Retreat</t>
-  </si>
-  <si>
-    <t>Photos by A. Park et al.</t>
-  </si>
-  <si>
     <t>placeholder-2.svg</t>
   </si>
   <si>
@@ -3561,6 +3558,18 @@
   </si>
   <si>
     <t>https://scholar.google.com/citations?user=-kIZuiIWuaUC&amp;hl=en</t>
+  </si>
+  <si>
+    <t>Our new lab website is live!</t>
+  </si>
+  <si>
+    <t>Welcome to the new home of the Pombo lab. Here you can find our latest research, publications, team members, and news. Stay tuned for updates!</t>
+  </si>
+  <si>
+    <t>Photos by A. Park</t>
+  </si>
+  <si>
+    <t>Sample</t>
   </si>
 </sst>
 </file>
@@ -4246,37 +4255,37 @@
   <sheetData>
     <row r="1" spans="1:12" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>96</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>463</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>464</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>465</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>466</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>467</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>145</v>
       </c>
       <c r="I1" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="K1" s="4" t="s">
         <v>468</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>469</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>470</v>
       </c>
       <c r="L1" s="4" t="s">
         <v>112</v>
@@ -4287,19 +4296,19 @@
         <v>2026</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>471</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>472</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>473</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>475</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>135</v>
@@ -4313,16 +4322,16 @@
         <v>2026</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>474</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>477</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>479</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>135</v>
@@ -4336,16 +4345,16 @@
         <v>2026</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>479</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>480</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>481</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>482</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>483</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>135</v>
@@ -4359,16 +4368,16 @@
         <v>2026</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>484</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>485</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>486</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>135</v>
@@ -4382,16 +4391,16 @@
         <v>2025</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>487</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>488</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>489</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>135</v>
@@ -4405,19 +4414,19 @@
         <v>2025</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>492</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>493</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>494</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>135</v>
@@ -4431,19 +4440,19 @@
         <v>2025</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>497</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>498</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>499</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>114</v>
@@ -4457,16 +4466,16 @@
         <v>2025</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>501</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>502</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>503</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>135</v>
@@ -4480,22 +4489,22 @@
         <v>2024</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>504</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>507</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>508</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>509</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>135</v>
@@ -4509,19 +4518,19 @@
         <v>2024</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>510</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>511</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>512</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>513</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>514</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>135</v>
@@ -4535,16 +4544,16 @@
         <v>2024</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>515</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>516</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>517</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>135</v>
@@ -4558,16 +4567,16 @@
         <v>2024</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>518</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>519</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>520</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>521</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>135</v>
@@ -4581,16 +4590,16 @@
         <v>2024</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>523</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>525</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>135</v>
@@ -4604,19 +4613,19 @@
         <v>2023</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>528</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>529</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>530</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>135</v>
@@ -4630,19 +4639,19 @@
         <v>2023</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>531</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>532</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>534</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>114</v>
@@ -4656,19 +4665,19 @@
         <v>2023</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>536</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>537</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>539</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>135</v>
@@ -4682,19 +4691,19 @@
         <v>2022</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>538</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>540</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>541</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>542</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>543</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>544</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>135</v>
@@ -4708,19 +4717,19 @@
         <v>2022</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>545</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>546</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>547</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>548</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>135</v>
@@ -4734,19 +4743,19 @@
         <v>2022</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>548</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>549</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>550</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>552</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>553</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>554</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>135</v>
@@ -4760,19 +4769,19 @@
         <v>2021</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>553</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>556</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="F21" s="2" t="s">
         <v>557</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>558</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>559</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>135</v>
@@ -4786,19 +4795,19 @@
         <v>2021</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>558</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>560</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>561</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>562</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>563</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>135</v>
@@ -4812,19 +4821,19 @@
         <v>2021</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>562</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="F23" s="2" t="s">
         <v>565</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>528</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>567</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>135</v>
@@ -4838,19 +4847,19 @@
         <v>2021</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="F24" s="2" t="s">
         <v>570</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>571</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>572</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>135</v>
@@ -4864,19 +4873,19 @@
         <v>2020</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E25" s="2" t="s">
         <v>573</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="F25" s="2" t="s">
         <v>574</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>575</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>576</v>
       </c>
       <c r="K25" s="2" t="s">
         <v>135</v>
@@ -4890,19 +4899,19 @@
         <v>2020</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>575</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>576</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>577</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="E26" s="2" t="s">
         <v>578</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>579</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>580</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>581</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>135</v>
@@ -4916,19 +4925,19 @@
         <v>2020</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>580</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>582</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="E27" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="F27" s="2" t="s">
         <v>584</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>585</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>586</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>135</v>
@@ -4942,19 +4951,19 @@
         <v>2020</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="E28" s="2" t="s">
         <v>588</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>589</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>590</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>591</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>135</v>
@@ -4968,19 +4977,19 @@
         <v>2019</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>591</v>
+      </c>
+      <c r="D29" s="2" t="s">
         <v>592</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="E29" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>594</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>596</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>135</v>
@@ -4994,19 +5003,19 @@
         <v>2019</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>596</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>597</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="F30" s="2" t="s">
         <v>598</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>600</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>135</v>
@@ -5020,19 +5029,19 @@
         <v>2018</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>600</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>601</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="E31" s="2" t="s">
         <v>602</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>603</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>605</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>135</v>
@@ -5046,19 +5055,19 @@
         <v>2018</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="F32" s="2" t="s">
         <v>607</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>603</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>608</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>609</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>135</v>
@@ -5072,19 +5081,19 @@
         <v>2017</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>611</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>612</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>613</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>135</v>
@@ -5098,19 +5107,19 @@
         <v>2017</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>612</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>613</v>
+      </c>
+      <c r="D34" s="2" t="s">
         <v>614</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="E34" s="2" t="s">
         <v>615</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="F34" s="2" t="s">
         <v>616</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>617</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>618</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>135</v>
@@ -5124,19 +5133,19 @@
         <v>2017</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>619</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="F35" s="2" t="s">
         <v>620</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>621</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>622</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>135</v>
@@ -5150,19 +5159,19 @@
         <v>2017</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>621</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="F36" s="2" t="s">
         <v>624</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>524</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>625</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>626</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>135</v>
@@ -5176,19 +5185,19 @@
         <v>2017</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>627</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="E37" s="2" t="s">
         <v>628</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>629</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>630</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>631</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>135</v>
@@ -5202,19 +5211,19 @@
         <v>2017</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>632</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="E38" s="2" t="s">
         <v>633</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="F38" s="2" t="s">
         <v>634</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>636</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>135</v>
@@ -5228,19 +5237,19 @@
         <v>2017</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>637</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="E39" s="2" t="s">
         <v>638</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="F39" s="2" t="s">
         <v>639</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>640</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>641</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>135</v>
@@ -5254,19 +5263,19 @@
         <v>2017</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>640</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>641</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E40" s="2" t="s">
         <v>642</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="F40" s="2" t="s">
         <v>643</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>644</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>645</v>
       </c>
       <c r="K40" s="2" t="s">
         <v>114</v>
@@ -5280,19 +5289,19 @@
         <v>2017</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>646</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="F41" s="2" t="s">
         <v>647</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>648</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>649</v>
       </c>
       <c r="K41" s="2" t="s">
         <v>135</v>
@@ -5306,19 +5315,19 @@
         <v>2016</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="E42" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="D42" s="2" t="s">
+      <c r="F42" s="2" t="s">
         <v>651</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>652</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>653</v>
       </c>
       <c r="K42" s="2" t="s">
         <v>135</v>
@@ -5332,19 +5341,19 @@
         <v>2016</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="E43" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="F43" s="2" t="s">
         <v>655</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>656</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>657</v>
       </c>
       <c r="K43" s="2" t="s">
         <v>135</v>
@@ -5358,19 +5367,19 @@
         <v>2016</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="E44" s="2" t="s">
         <v>658</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>620</v>
-      </c>
-      <c r="D44" s="2" t="s">
+      <c r="F44" s="2" t="s">
         <v>659</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>661</v>
       </c>
       <c r="K44" s="2" t="s">
         <v>135</v>
@@ -5384,19 +5393,19 @@
         <v>2016</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>662</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="E45" s="2" t="s">
         <v>663</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="F45" s="2" t="s">
         <v>664</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>665</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>666</v>
       </c>
       <c r="K45" s="2" t="s">
         <v>135</v>
@@ -5410,19 +5419,19 @@
         <v>2015</v>
       </c>
       <c r="B46" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>667</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="E46" s="2" t="s">
         <v>668</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="F46" s="2" t="s">
         <v>669</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>671</v>
       </c>
       <c r="K46" s="2" t="s">
         <v>135</v>
@@ -5436,19 +5445,19 @@
         <v>2015</v>
       </c>
       <c r="B47" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="E47" s="2" t="s">
         <v>672</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="F47" s="2" t="s">
         <v>673</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>497</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>674</v>
-      </c>
-      <c r="F47" s="2" t="s">
-        <v>675</v>
       </c>
       <c r="K47" s="2" t="s">
         <v>135</v>
@@ -5462,19 +5471,19 @@
         <v>2015</v>
       </c>
       <c r="B48" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>676</v>
       </c>
-      <c r="C48" s="2" t="s">
+      <c r="E48" s="2" t="s">
         <v>677</v>
       </c>
-      <c r="D48" s="2" t="s">
+      <c r="F48" s="2" t="s">
         <v>678</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>679</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>680</v>
       </c>
       <c r="K48" s="2" t="s">
         <v>135</v>
@@ -5488,19 +5497,19 @@
         <v>2015</v>
       </c>
       <c r="B49" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>680</v>
+      </c>
+      <c r="D49" s="2" t="s">
         <v>681</v>
       </c>
-      <c r="C49" s="2" t="s">
+      <c r="E49" s="2" t="s">
         <v>682</v>
       </c>
-      <c r="D49" s="2" t="s">
+      <c r="F49" s="2" t="s">
         <v>683</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>684</v>
-      </c>
-      <c r="F49" s="2" t="s">
-        <v>685</v>
       </c>
       <c r="K49" s="2" t="s">
         <v>135</v>
@@ -5514,19 +5523,19 @@
         <v>2015</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="E50" s="2" t="s">
         <v>686</v>
       </c>
-      <c r="C50" s="2" t="s">
+      <c r="F50" s="2" t="s">
         <v>687</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>542</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>688</v>
-      </c>
-      <c r="F50" s="2" t="s">
-        <v>689</v>
       </c>
       <c r="K50" s="2" t="s">
         <v>135</v>
@@ -5540,19 +5549,19 @@
         <v>2014</v>
       </c>
       <c r="B51" s="2" t="s">
+        <v>688</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>689</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="E51" s="2" t="s">
         <v>690</v>
       </c>
-      <c r="C51" s="2" t="s">
+      <c r="F51" s="2" t="s">
         <v>691</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>692</v>
-      </c>
-      <c r="F51" s="2" t="s">
-        <v>693</v>
       </c>
       <c r="K51" s="2" t="s">
         <v>135</v>
@@ -5566,19 +5575,19 @@
         <v>2014</v>
       </c>
       <c r="B52" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>693</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="E52" s="2" t="s">
         <v>694</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="F52" s="2" t="s">
         <v>695</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>696</v>
-      </c>
-      <c r="F52" s="2" t="s">
-        <v>697</v>
       </c>
       <c r="K52" s="2" t="s">
         <v>135</v>
@@ -5592,19 +5601,19 @@
         <v>2014</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>698</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="E53" s="2" t="s">
         <v>699</v>
       </c>
-      <c r="D53" s="2" t="s">
+      <c r="F53" s="2" t="s">
         <v>700</v>
-      </c>
-      <c r="E53" s="2" t="s">
-        <v>701</v>
-      </c>
-      <c r="F53" s="2" t="s">
-        <v>702</v>
       </c>
       <c r="K53" s="2" t="s">
         <v>135</v>
@@ -5618,19 +5627,19 @@
         <v>2014</v>
       </c>
       <c r="B54" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>703</v>
       </c>
-      <c r="C54" s="2" t="s">
+      <c r="E54" s="2" t="s">
         <v>704</v>
       </c>
-      <c r="D54" s="2" t="s">
+      <c r="F54" s="2" t="s">
         <v>705</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>706</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>707</v>
       </c>
       <c r="K54" s="2" t="s">
         <v>135</v>
@@ -5644,19 +5653,19 @@
         <v>2013</v>
       </c>
       <c r="B55" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>707</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>708</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="E55" s="2" t="s">
         <v>709</v>
       </c>
-      <c r="D55" s="2" t="s">
+      <c r="F55" s="2" t="s">
         <v>710</v>
-      </c>
-      <c r="E55" s="2" t="s">
-        <v>711</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>712</v>
       </c>
       <c r="K55" s="2" t="s">
         <v>135</v>
@@ -5670,19 +5679,19 @@
         <v>2013</v>
       </c>
       <c r="B56" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>712</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>713</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="E56" s="2" t="s">
         <v>714</v>
       </c>
-      <c r="D56" s="2" t="s">
+      <c r="F56" s="2" t="s">
         <v>715</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>716</v>
-      </c>
-      <c r="F56" s="2" t="s">
-        <v>717</v>
       </c>
       <c r="K56" s="2" t="s">
         <v>135</v>
@@ -5696,19 +5705,19 @@
         <v>2013</v>
       </c>
       <c r="B57" s="2" t="s">
+        <v>716</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>717</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>718</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="E57" s="2" t="s">
         <v>719</v>
       </c>
-      <c r="D57" s="2" t="s">
+      <c r="F57" s="2" t="s">
         <v>720</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>721</v>
-      </c>
-      <c r="F57" s="2" t="s">
-        <v>722</v>
       </c>
       <c r="K57" s="2" t="s">
         <v>135</v>
@@ -5722,19 +5731,19 @@
         <v>2013</v>
       </c>
       <c r="B58" s="2" t="s">
+        <v>721</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>723</v>
       </c>
-      <c r="C58" s="2" t="s">
+      <c r="E58" s="2" t="s">
         <v>724</v>
       </c>
-      <c r="D58" s="2" t="s">
+      <c r="F58" s="2" t="s">
         <v>725</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>726</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>727</v>
       </c>
       <c r="K58" s="2" t="s">
         <v>135</v>
@@ -5748,19 +5757,19 @@
         <v>2012</v>
       </c>
       <c r="B59" s="2" t="s">
+        <v>726</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>727</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>728</v>
       </c>
-      <c r="C59" s="2" t="s">
+      <c r="E59" s="2" t="s">
         <v>729</v>
       </c>
-      <c r="D59" s="2" t="s">
+      <c r="F59" s="2" t="s">
         <v>730</v>
-      </c>
-      <c r="E59" s="2" t="s">
-        <v>731</v>
-      </c>
-      <c r="F59" s="2" t="s">
-        <v>732</v>
       </c>
       <c r="K59" s="2" t="s">
         <v>135</v>
@@ -5774,19 +5783,19 @@
         <v>2012</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>731</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>732</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>733</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>724</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>734</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>735</v>
       </c>
       <c r="K60" s="2" t="s">
         <v>135</v>
@@ -5800,19 +5809,19 @@
         <v>2012</v>
       </c>
       <c r="B61" s="2" t="s">
+        <v>734</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>736</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="E61" s="2" t="s">
         <v>737</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="F61" s="2" t="s">
         <v>738</v>
-      </c>
-      <c r="E61" s="2" t="s">
-        <v>739</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>740</v>
       </c>
       <c r="K61" s="2" t="s">
         <v>135</v>
@@ -5826,19 +5835,19 @@
         <v>2012</v>
       </c>
       <c r="B62" s="2" t="s">
+        <v>739</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>741</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="E62" s="2" t="s">
         <v>742</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="F62" s="2" t="s">
         <v>743</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>744</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>745</v>
       </c>
       <c r="K62" s="2" t="s">
         <v>135</v>
@@ -5852,19 +5861,19 @@
         <v>2012</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>744</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>745</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="E63" s="2" t="s">
         <v>746</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="F63" s="2" t="s">
         <v>747</v>
-      </c>
-      <c r="D63" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="E63" s="2" t="s">
-        <v>748</v>
-      </c>
-      <c r="F63" s="2" t="s">
-        <v>749</v>
       </c>
       <c r="K63" s="2" t="s">
         <v>135</v>
@@ -5878,19 +5887,19 @@
         <v>2011</v>
       </c>
       <c r="B64" s="2" t="s">
+        <v>748</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>749</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>750</v>
       </c>
-      <c r="C64" s="2" t="s">
+      <c r="E64" s="2" t="s">
         <v>751</v>
       </c>
-      <c r="D64" s="2" t="s">
+      <c r="F64" s="2" t="s">
         <v>752</v>
-      </c>
-      <c r="E64" s="2" t="s">
-        <v>753</v>
-      </c>
-      <c r="F64" s="2" t="s">
-        <v>754</v>
       </c>
       <c r="K64" s="2" t="s">
         <v>135</v>
@@ -5904,19 +5913,19 @@
         <v>2011</v>
       </c>
       <c r="B65" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>754</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="E65" s="2" t="s">
         <v>755</v>
       </c>
-      <c r="C65" s="2" t="s">
+      <c r="F65" s="2" t="s">
         <v>756</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="E65" s="2" t="s">
-        <v>757</v>
-      </c>
-      <c r="F65" s="2" t="s">
-        <v>758</v>
       </c>
       <c r="K65" s="2" t="s">
         <v>135</v>
@@ -5930,19 +5939,19 @@
         <v>2010</v>
       </c>
       <c r="B66" s="2" t="s">
+        <v>757</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>758</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>759</v>
       </c>
-      <c r="C66" s="2" t="s">
+      <c r="E66" s="2" t="s">
         <v>760</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="F66" s="2" t="s">
         <v>761</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>762</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>763</v>
       </c>
       <c r="K66" s="2" t="s">
         <v>135</v>
@@ -5956,19 +5965,19 @@
         <v>2010</v>
       </c>
       <c r="B67" s="2" t="s">
+        <v>762</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>763</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="E67" s="2" t="s">
         <v>764</v>
       </c>
-      <c r="C67" s="2" t="s">
+      <c r="F67" s="2" t="s">
         <v>765</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>512</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>766</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>767</v>
       </c>
       <c r="K67" s="2" t="s">
         <v>135</v>
@@ -5982,19 +5991,19 @@
         <v>2010</v>
       </c>
       <c r="B68" s="2" t="s">
+        <v>766</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>767</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>768</v>
       </c>
-      <c r="C68" s="2" t="s">
+      <c r="E68" s="2" t="s">
         <v>769</v>
       </c>
-      <c r="D68" s="2" t="s">
+      <c r="F68" s="2" t="s">
         <v>770</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>771</v>
-      </c>
-      <c r="F68" s="2" t="s">
-        <v>772</v>
       </c>
       <c r="K68" s="2" t="s">
         <v>135</v>
@@ -6008,19 +6017,19 @@
         <v>2010</v>
       </c>
       <c r="B69" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>772</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="E69" s="2" t="s">
         <v>773</v>
       </c>
-      <c r="C69" s="2" t="s">
+      <c r="F69" s="2" t="s">
         <v>774</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>664</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>775</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>776</v>
       </c>
       <c r="K69" s="2" t="s">
         <v>135</v>
@@ -6034,19 +6043,19 @@
         <v>2010</v>
       </c>
       <c r="B70" s="2" t="s">
+        <v>775</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>776</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="E70" s="2" t="s">
         <v>777</v>
       </c>
-      <c r="C70" s="2" t="s">
+      <c r="F70" s="2" t="s">
         <v>778</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>779</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>780</v>
       </c>
       <c r="K70" s="2" t="s">
         <v>135</v>
@@ -6060,19 +6069,19 @@
         <v>2010</v>
       </c>
       <c r="B71" s="2" t="s">
+        <v>779</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>780</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>781</v>
       </c>
-      <c r="C71" s="2" t="s">
+      <c r="E71" s="2" t="s">
         <v>782</v>
       </c>
-      <c r="D71" s="2" t="s">
+      <c r="F71" s="2" t="s">
         <v>783</v>
-      </c>
-      <c r="E71" s="2" t="s">
-        <v>784</v>
-      </c>
-      <c r="F71" s="2" t="s">
-        <v>785</v>
       </c>
       <c r="K71" s="2" t="s">
         <v>135</v>
@@ -6086,19 +6095,19 @@
         <v>2010</v>
       </c>
       <c r="B72" s="2" t="s">
+        <v>784</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>785</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>786</v>
       </c>
-      <c r="C72" s="2" t="s">
+      <c r="E72" s="2" t="s">
         <v>787</v>
       </c>
-      <c r="D72" s="2" t="s">
+      <c r="F72" s="2" t="s">
         <v>788</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>789</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>790</v>
       </c>
       <c r="K72" s="2" t="s">
         <v>135</v>
@@ -6112,19 +6121,19 @@
         <v>2010</v>
       </c>
       <c r="B73" s="2" t="s">
+        <v>789</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>790</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>791</v>
       </c>
-      <c r="C73" s="2" t="s">
+      <c r="E73" s="2" t="s">
         <v>792</v>
       </c>
-      <c r="D73" s="2" t="s">
+      <c r="F73" s="2" t="s">
         <v>793</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>794</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>795</v>
       </c>
       <c r="K73" s="2" t="s">
         <v>135</v>
@@ -6138,19 +6147,19 @@
         <v>2009</v>
       </c>
       <c r="B74" s="2" t="s">
+        <v>794</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>795</v>
+      </c>
+      <c r="D74" s="2" t="s">
         <v>796</v>
       </c>
-      <c r="C74" s="2" t="s">
+      <c r="E74" s="2" t="s">
         <v>797</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="F74" s="2" t="s">
         <v>798</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>799</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>800</v>
       </c>
       <c r="K74" s="2" t="s">
         <v>135</v>
@@ -6164,19 +6173,19 @@
         <v>2009</v>
       </c>
       <c r="B75" s="2" t="s">
+        <v>799</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>740</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="E75" s="2" t="s">
         <v>801</v>
       </c>
-      <c r="C75" s="2" t="s">
-        <v>742</v>
-      </c>
-      <c r="D75" s="2" t="s">
+      <c r="F75" s="2" t="s">
         <v>802</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>803</v>
-      </c>
-      <c r="F75" s="2" t="s">
-        <v>804</v>
       </c>
       <c r="K75" s="2" t="s">
         <v>135</v>
@@ -6190,19 +6199,19 @@
         <v>2009</v>
       </c>
       <c r="B76" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>804</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="E76" s="2" t="s">
         <v>805</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="F76" s="2" t="s">
         <v>806</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>651</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>807</v>
-      </c>
-      <c r="F76" s="2" t="s">
-        <v>808</v>
       </c>
       <c r="K76" s="2" t="s">
         <v>135</v>
@@ -6216,19 +6225,19 @@
         <v>2009</v>
       </c>
       <c r="B77" s="2" t="s">
+        <v>807</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>808</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>809</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="E77" s="2" t="s">
         <v>810</v>
       </c>
-      <c r="D77" s="2" t="s">
+      <c r="F77" s="2" t="s">
         <v>811</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>812</v>
-      </c>
-      <c r="F77" s="2" t="s">
-        <v>813</v>
       </c>
       <c r="K77" s="2" t="s">
         <v>135</v>
@@ -6242,19 +6251,19 @@
         <v>2008</v>
       </c>
       <c r="B78" s="2" t="s">
+        <v>812</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>813</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E78" s="2" t="s">
         <v>814</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="F78" s="2" t="s">
         <v>815</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>816</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>817</v>
       </c>
       <c r="K78" s="2" t="s">
         <v>135</v>
@@ -6268,19 +6277,19 @@
         <v>2008</v>
       </c>
       <c r="B79" s="2" t="s">
+        <v>816</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="D79" s="2" t="s">
         <v>818</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="E79" s="2" t="s">
         <v>819</v>
       </c>
-      <c r="D79" s="2" t="s">
+      <c r="F79" s="2" t="s">
         <v>820</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>821</v>
-      </c>
-      <c r="F79" s="2" t="s">
-        <v>822</v>
       </c>
       <c r="K79" s="2" t="s">
         <v>135</v>
@@ -6294,19 +6303,19 @@
         <v>2008</v>
       </c>
       <c r="B80" s="2" t="s">
+        <v>821</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>822</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>750</v>
+      </c>
+      <c r="E80" s="2" t="s">
         <v>823</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="F80" s="2" t="s">
         <v>824</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>752</v>
-      </c>
-      <c r="E80" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="F80" s="2" t="s">
-        <v>826</v>
       </c>
       <c r="K80" s="2" t="s">
         <v>135</v>
@@ -6320,19 +6329,19 @@
         <v>2007</v>
       </c>
       <c r="B81" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="D81" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="E81" s="2" t="s">
         <v>827</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="F81" s="2" t="s">
         <v>828</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>664</v>
-      </c>
-      <c r="E81" s="2" t="s">
-        <v>829</v>
-      </c>
-      <c r="F81" s="2" t="s">
-        <v>830</v>
       </c>
       <c r="K81" s="2" t="s">
         <v>135</v>
@@ -6346,19 +6355,19 @@
         <v>2007</v>
       </c>
       <c r="B82" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="C82" s="2" t="s">
+        <v>830</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E82" s="2" t="s">
         <v>831</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="F82" s="2" t="s">
         <v>832</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>570</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>833</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>834</v>
       </c>
       <c r="K82" s="2" t="s">
         <v>135</v>
@@ -6372,19 +6381,19 @@
         <v>2007</v>
       </c>
       <c r="B83" s="2" t="s">
+        <v>833</v>
+      </c>
+      <c r="C83" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>835</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="E83" s="2" t="s">
         <v>836</v>
       </c>
-      <c r="D83" s="2" t="s">
+      <c r="F83" s="2" t="s">
         <v>837</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>838</v>
-      </c>
-      <c r="F83" s="2" t="s">
-        <v>839</v>
       </c>
       <c r="K83" s="2" t="s">
         <v>135</v>
@@ -6398,19 +6407,19 @@
         <v>2007</v>
       </c>
       <c r="B84" s="2" t="s">
+        <v>838</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>839</v>
+      </c>
+      <c r="D84" s="2" t="s">
         <v>840</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="E84" s="2" t="s">
         <v>841</v>
       </c>
-      <c r="D84" s="2" t="s">
+      <c r="F84" s="2" t="s">
         <v>842</v>
-      </c>
-      <c r="E84" s="2" t="s">
-        <v>843</v>
-      </c>
-      <c r="F84" s="2" t="s">
-        <v>844</v>
       </c>
       <c r="K84" s="2" t="s">
         <v>135</v>
@@ -6424,19 +6433,19 @@
         <v>2007</v>
       </c>
       <c r="B85" s="2" t="s">
+        <v>843</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>844</v>
+      </c>
+      <c r="D85" s="2" t="s">
         <v>845</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="E85" s="2" t="s">
         <v>846</v>
       </c>
-      <c r="D85" s="2" t="s">
+      <c r="F85" s="2" t="s">
         <v>847</v>
-      </c>
-      <c r="E85" s="2" t="s">
-        <v>848</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>849</v>
       </c>
       <c r="K85" s="2" t="s">
         <v>135</v>
@@ -6450,19 +6459,19 @@
         <v>2006</v>
       </c>
       <c r="B86" s="2" t="s">
+        <v>848</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>844</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>781</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>849</v>
+      </c>
+      <c r="F86" s="2" t="s">
         <v>850</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>846</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>783</v>
-      </c>
-      <c r="E86" s="2" t="s">
-        <v>851</v>
-      </c>
-      <c r="F86" s="2" t="s">
-        <v>852</v>
       </c>
       <c r="K86" s="2" t="s">
         <v>135</v>
@@ -6476,19 +6485,19 @@
         <v>2006</v>
       </c>
       <c r="B87" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="E87" s="2" t="s">
         <v>853</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="F87" s="2" t="s">
         <v>854</v>
-      </c>
-      <c r="D87" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>855</v>
-      </c>
-      <c r="F87" s="2" t="s">
-        <v>856</v>
       </c>
       <c r="K87" s="2" t="s">
         <v>135</v>
@@ -6502,19 +6511,19 @@
         <v>2006</v>
       </c>
       <c r="B88" s="2" t="s">
+        <v>855</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>856</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>835</v>
+      </c>
+      <c r="E88" s="2" t="s">
         <v>857</v>
       </c>
-      <c r="C88" s="2" t="s">
+      <c r="F88" s="2" t="s">
         <v>858</v>
-      </c>
-      <c r="D88" s="2" t="s">
-        <v>837</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>859</v>
-      </c>
-      <c r="F88" s="2" t="s">
-        <v>860</v>
       </c>
       <c r="K88" s="2" t="s">
         <v>135</v>
@@ -6528,19 +6537,19 @@
         <v>2005</v>
       </c>
       <c r="B89" s="2" t="s">
+        <v>859</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>860</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="E89" s="2" t="s">
         <v>861</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="F89" s="2" t="s">
         <v>862</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>802</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>863</v>
-      </c>
-      <c r="F89" s="2" t="s">
-        <v>864</v>
       </c>
       <c r="K89" s="2" t="s">
         <v>135</v>
@@ -6554,19 +6563,19 @@
         <v>2005</v>
       </c>
       <c r="B90" s="2" t="s">
+        <v>863</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>864</v>
+      </c>
+      <c r="D90" s="2" t="s">
         <v>865</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="E90" s="2" t="s">
         <v>866</v>
       </c>
-      <c r="D90" s="2" t="s">
+      <c r="F90" s="2" t="s">
         <v>867</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>868</v>
-      </c>
-      <c r="F90" s="2" t="s">
-        <v>869</v>
       </c>
       <c r="K90" s="2" t="s">
         <v>135</v>
@@ -6580,19 +6589,19 @@
         <v>2004</v>
       </c>
       <c r="B91" s="2" t="s">
+        <v>868</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>869</v>
+      </c>
+      <c r="D91" s="2" t="s">
         <v>870</v>
       </c>
-      <c r="C91" s="2" t="s">
+      <c r="E91" s="2" t="s">
         <v>871</v>
       </c>
-      <c r="D91" s="2" t="s">
+      <c r="F91" s="2" t="s">
         <v>872</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>873</v>
-      </c>
-      <c r="F91" s="2" t="s">
-        <v>874</v>
       </c>
       <c r="K91" s="2" t="s">
         <v>135</v>
@@ -6606,19 +6615,19 @@
         <v>2004</v>
       </c>
       <c r="B92" s="2" t="s">
+        <v>873</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="D92" s="2" t="s">
         <v>875</v>
       </c>
-      <c r="C92" s="2" t="s">
+      <c r="E92" s="2" t="s">
         <v>876</v>
       </c>
-      <c r="D92" s="2" t="s">
+      <c r="F92" s="2" t="s">
         <v>877</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>878</v>
-      </c>
-      <c r="F92" s="2" t="s">
-        <v>879</v>
       </c>
       <c r="K92" s="2" t="s">
         <v>135</v>
@@ -6632,19 +6641,19 @@
         <v>2004</v>
       </c>
       <c r="B93" s="2" t="s">
+        <v>878</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>879</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="E93" s="2" t="s">
         <v>880</v>
       </c>
-      <c r="C93" s="2" t="s">
+      <c r="F93" s="2" t="s">
         <v>881</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="E93" s="2" t="s">
-        <v>882</v>
-      </c>
-      <c r="F93" s="2" t="s">
-        <v>883</v>
       </c>
       <c r="K93" s="2" t="s">
         <v>135</v>
@@ -6658,19 +6667,19 @@
         <v>2003</v>
       </c>
       <c r="B94" s="2" t="s">
+        <v>882</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>883</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>884</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="E94" s="2" t="s">
         <v>885</v>
       </c>
-      <c r="D94" s="2" t="s">
+      <c r="F94" s="2" t="s">
         <v>886</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>887</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>888</v>
       </c>
       <c r="K94" s="2" t="s">
         <v>135</v>
@@ -6684,19 +6693,19 @@
         <v>2003</v>
       </c>
       <c r="B95" s="2" t="s">
+        <v>887</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>888</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>818</v>
+      </c>
+      <c r="E95" s="2" t="s">
         <v>889</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="F95" s="2" t="s">
         <v>890</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>820</v>
-      </c>
-      <c r="E95" s="2" t="s">
-        <v>891</v>
-      </c>
-      <c r="F95" s="2" t="s">
-        <v>892</v>
       </c>
       <c r="K95" s="2" t="s">
         <v>135</v>
@@ -6710,19 +6719,19 @@
         <v>2003</v>
       </c>
       <c r="B96" s="2" t="s">
+        <v>891</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>892</v>
+      </c>
+      <c r="D96" s="2" t="s">
         <v>893</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="E96" s="2" t="s">
         <v>894</v>
       </c>
-      <c r="D96" s="2" t="s">
+      <c r="F96" s="2" t="s">
         <v>895</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>896</v>
-      </c>
-      <c r="F96" s="2" t="s">
-        <v>897</v>
       </c>
       <c r="K96" s="2" t="s">
         <v>135</v>
@@ -6736,19 +6745,19 @@
         <v>2003</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="D97" s="2" t="s">
         <v>60</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="K97" s="2" t="s">
         <v>135</v>
@@ -6762,19 +6771,19 @@
         <v>2003</v>
       </c>
       <c r="B98" s="2" t="s">
+        <v>900</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>834</v>
+      </c>
+      <c r="D98" s="2" t="s">
+        <v>901</v>
+      </c>
+      <c r="E98" s="2" t="s">
         <v>902</v>
       </c>
-      <c r="C98" s="2" t="s">
-        <v>836</v>
-      </c>
-      <c r="D98" s="2" t="s">
+      <c r="F98" s="2" t="s">
         <v>903</v>
-      </c>
-      <c r="E98" s="2" t="s">
-        <v>904</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>905</v>
       </c>
       <c r="K98" s="2" t="s">
         <v>135</v>
@@ -6788,19 +6797,19 @@
         <v>2003</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="D99" s="2" t="s">
         <v>60</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="F99" s="2" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="K99" s="2" t="s">
         <v>135</v>
@@ -6841,22 +6850,22 @@
   <sheetData>
     <row r="1" spans="1:8" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>96</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>908</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>909</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>910</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>911</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>912</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>913</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>111</v>
@@ -6870,19 +6879,19 @@
         <v>2026</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>913</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>914</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>915</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>916</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>917</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>918</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>135</v>
@@ -6893,19 +6902,19 @@
         <v>2025</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>913</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>914</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>915</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
+        <v>917</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>916</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>919</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>918</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>135</v>
@@ -6997,7 +7006,7 @@
         <v>62</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>63</v>
@@ -7728,19 +7737,19 @@
     </row>
     <row r="3" spans="1:9" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>152</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>114</v>
@@ -7754,10 +7763,10 @@
         <v>152</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>176</v>
@@ -7777,7 +7786,7 @@
         <v>178</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>179</v>
@@ -7812,7 +7821,7 @@
         <v>186</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>114</v>
@@ -7884,7 +7893,7 @@
         <v>184</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>197</v>
@@ -7904,7 +7913,7 @@
         <v>231</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>199</v>
@@ -7927,7 +7936,7 @@
         <v>172</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>229</v>
@@ -7947,16 +7956,16 @@
         <v>231</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>232</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>114</v>
@@ -7970,10 +7979,10 @@
         <v>157</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>925</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>927</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>929</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>236</v>
@@ -7984,7 +7993,7 @@
     </row>
     <row r="14" spans="1:9" s="2" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>157</v>
@@ -7993,7 +8002,7 @@
         <v>231</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="32" x14ac:dyDescent="0.2">
@@ -8007,7 +8016,7 @@
         <v>202</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
@@ -8032,7 +8041,7 @@
         <v>172</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
@@ -8054,10 +8063,10 @@
         <v>157</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>234</v>
@@ -8077,7 +8086,7 @@
         <v>231</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
@@ -8104,7 +8113,7 @@
         <v>172</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
@@ -8129,7 +8138,7 @@
         <v>178</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
@@ -8154,7 +8163,7 @@
         <v>172</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
@@ -8179,7 +8188,7 @@
         <v>231</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>222</v>
@@ -8199,16 +8208,16 @@
     </row>
     <row r="23" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>157</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
@@ -8229,7 +8238,7 @@
         <v>231</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -8237,7 +8246,7 @@
         <v>227</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>114</v>
@@ -9468,7 +9477,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" style="7" customWidth="1"/>
@@ -9498,227 +9507,244 @@
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="9">
+        <v>46302</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>935</v>
+      </c>
+      <c r="D2" t="s">
+        <v>936</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A3" s="9">
         <v>46212</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="2" customFormat="1" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="9">
+      <c r="F3" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="2" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" s="9">
         <v>46175</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
-      <c r="A4" s="9">
-        <v>45938</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>413</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
-        <v>45799</v>
+        <v>45938</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
-        <v>45637</v>
+        <v>45799</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
-        <v>45333</v>
+        <v>45637</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
-        <v>45096</v>
+        <v>45333</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>425</v>
+        <v>407</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
+        <v>45096</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A10" s="9">
         <v>44980</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>429</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>430</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
-      <c r="A10" s="9">
+      <c r="F10" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="2" customFormat="1" ht="64" x14ac:dyDescent="0.2">
+      <c r="A11" s="9">
         <v>44517</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>434</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
-      <c r="A11" s="9">
-        <v>44120</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>437</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
+        <v>44120</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="2" customFormat="1" ht="48" x14ac:dyDescent="0.2">
+      <c r="A13" s="9">
         <v>43766</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>440</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>114</v>
+      <c r="F13" s="2" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Show" error="Set to &quot;no&quot; to hide this row on the website without deleting it." sqref="F2:F1000" xr:uid="{00000000-0002-0000-0700-000000000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Show" error="Set to &quot;no&quot; to hide this row on the website without deleting it." sqref="F2:F1001" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9765,24 +9791,24 @@
         <v>444</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>445</v>
+        <v>938</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>920</v>
+        <v>918</v>
       </c>
       <c r="D2" s="9">
         <v>46175</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>446</v>
+        <v>937</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="D3" s="9">
         <v>46156</v>
@@ -9793,19 +9819,19 @@
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>448</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>449</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>450</v>
       </c>
       <c r="D4" s="9">
         <v>46132</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>135</v>
@@ -9813,10 +9839,10 @@
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="D5" s="9">
         <v>46092</v>
@@ -9827,16 +9853,16 @@
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="D6" s="9">
         <v>45903</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>135</v>
@@ -9844,10 +9870,10 @@
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D7" s="9">
         <v>45644</v>
@@ -9858,7 +9884,7 @@
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="D8" s="9">
         <v>45598</v>
@@ -9869,10 +9895,10 @@
     </row>
     <row r="9" spans="1:6" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="D9" s="9">
         <v>45566</v>
@@ -9882,7 +9908,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
+  <autoFilter ref="A1:F9" xr:uid="{00000000-0009-0000-0000-000008000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Show" error="Set to &quot;no&quot; to hide this row on the website without deleting it." sqref="F2:F1000" xr:uid="{00000000-0002-0000-0800-000000000000}">
       <formula1>"yes,no"</formula1>

</xml_diff>